<commit_message>
WIP full v22 re-stamp: deliverables + spec_ref story fix + reports
76 non-automated WIP cases re-stamped v21->v22 (byte-verified), C30530 content
reword per v22 S11-R3 (HOLD kept), 10 automated held, C30456/C30464 spec_ref
story fix (SV-8654/8656 -> SV-8658/8659). id-map 508 (0 blanks), import header
sha256==peers, four counts set-equal, 0 foreign touched, run 359 untouched.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/Report-Suite_Work-In-Progress-Report_testrail-import.xlsx
+++ b/testrail-import/Report-Suite_Work-In-Progress-Report_testrail-import.xlsx
@@ -528,13 +528,13 @@
 2. Clicking it opens the Work In Progress report.
 3. The browser page title is exactly "Work In Progress - Report | ShopView" — a plain hyphen with one space on each side.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S1-R1, S1-R5), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S1-R1, S1-R5), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>SV-8657 (WIP spec v21 2026-08-17 Story 1 S1-R1; S1-R5 — S1-R5 CLOSES the page title verbatim; Performance group below the named anchor items per the PRD video 2026-07-30; access = the one ordinary reports permission per QA lead 2026-08-03)</t>
+          <t>SV-8657 (WIP spec v22 2026-08-18 Story 1 S1-R1; S1-R5 — S1-R5 CLOSES the page title verbatim; Performance group below the named anchor items per the PRD video 2026-07-30; access = the one ordinary reports permission per QA lead 2026-08-03)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
@@ -631,13 +631,13 @@
           <t>1. Only the four progress tabs exist — there is no Trend tab and no chart of work-in-progress dollars over time.
 2. No screen in the report reads or displays the nightly snapshot history.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S11-R7), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S11-R7), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>SV-8667 (WIP spec v21 2026-08-17 §2 Out of scope; §2 Known Limitations (v1); Story 11 S11-R7)</t>
+          <t>SV-8667 (WIP spec v22 2026-08-18 §2 Out of scope; §2 Known Limitations (v1); Story 11 S11-R7)</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
@@ -688,7 +688,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>SV-8654 (WIP spec v22 2026-08-17 S2-R4; S7-R7; population is work open on the as-of date,not filtered by created date)</t>
+          <t>SV-8658 (WIP spec v22 2026-08-17 S2-R4; S7-R7; population is work open on the as-of date,not filtered by created date)</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
@@ -735,13 +735,13 @@
 2. The part-sale work order does not appear anywhere either.
 3. No excluded work order's money is counted in any figure.
 ---
-This is the expected behaviour as per epic SV-8582 and the Work In Progress report specification version 21 (S2-R5), both read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S2-R5), read on 18 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>SV-8654 (WIP spec v21 2026-08-17 S2-R5; open work on the as-of date)</t>
+          <t>SV-8654 (WIP spec v22 2026-08-18 S2-R5; open work on the as-of date)</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr"/>
@@ -838,13 +838,13 @@
 2. The existing rows are replaced only when the new data returns (the table does not go blank and stay blank mid-load).
 3. Both a date-range change and a location change reload the report's rows.
 ---
-This is the expected behaviour as per epic SV-8582 and the Work In Progress report specification version 21 (S2-R6), both read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S2-R6), read on 18 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>SV-8655 (WIP spec v21 2026-08-17 S2-R6; changing the as-of date reloads)</t>
+          <t>SV-8655 (WIP spec v22 2026-08-18 S2-R6; changing the as-of date reloads)</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>SV-8656 (WIP spec v22 2026-08-17 S3; Approved started-boundary on the as-of date)</t>
+          <t>SV-8659 (WIP spec v22 2026-08-17 S3; Approved started-boundary on the as-of date)</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
@@ -1103,13 +1103,13 @@
 2. With all columns on, the full left-to-right order is: WO #, Status, Customer, Asset, VIN, Location, Advisor, Days Open, Last Activity, Labor Earned, Labor Remaining, Parts Earned, Parts Remaining, Earned, Remaining, Adjustments, Labor Delta, Total.
 3. "Adjustments" sits immediately before "Labor Delta" and "Total".
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and story SV-9282, and the Work In Progress report specification version 21 (S4-R1, S4-R2), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and story SV-9282, and the Work In Progress report specification version 22 (S4-R1, S4-R2), read on 18 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>SV-9282 (WIP spec v21 2026-08-14 S4-R1; S4-R2 — Adjustments column added; shared WIP+SBC proposal 2026-08-12)</t>
+          <t>SV-9282 (WIP spec v22 2026-08-18 S4-R1; S4-R2 — Adjustments column added; shared WIP+SBC proposal 2026-08-12)</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr"/>
@@ -1160,13 +1160,13 @@
 · If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 · If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582 and the Work In Progress report specification version 21 (S4-R1), both read on 17 August 2026. The column was renamed from "Inv. Hrs" to "Labor Delta" per SV-9071; only the name changed.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R1), read on 18 August 2026. The column was renamed from "Inv. Hrs" to "Labor Delta" per SV-9071; only the name changed.
 AUTOMATION: READY - EXPECT FAIL (SV-8987)</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 S4-R1; renamed to Labor Delta per SV-9071)</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 S4-R1; renamed to Labor Delta per SV-9071)</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
@@ -1217,13 +1217,13 @@
 - If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 - If it PASSES, the fix has shipped: tell the QA lead so this note can be removed.
 ---
-This is the expected behaviour as per epic SV-8582 and the Work In Progress report specification version 21 (S4-R2; S4-R3; S8-R3; S8-R4), both read on 17 August 2026. The column was renamed from "Inv. Hrs" to "Labor Delta" per SV-9071; only the name changed. Chris Ward confirmed this same Location rule in his answers of 10 August 2026 (build/report-suite/chris-answers-2026-08-10/), and the specification agrees (read on 10 August 2026).
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R2; S4-R3; S8-R3; S8-R4), read on 18 August 2026. The column was renamed from "Inv. Hrs" to "Labor Delta" per SV-9071; only the name changed. Chris Ward confirmed this same Location rule in his answers of 10 August 2026 (build/report-suite/chris-answers-2026-08-10/), and the specification agrees (read on 10 August 2026).
 AUTOMATION: HOLD - the build does not follow the ratified Location rule; the defect is written up in DEFECTS-FOR-PERMISSION.md and needs the QA lead's permission before a ticket exists to point at</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>SV-8660; SV-8664 (WIP spec v21 2026-08-17 S4-R2; S4-R3; S8-R3; S8-R4; renamed to Labor Delta per SV-9071)</t>
+          <t>SV-8660; SV-8664 (WIP spec v22 2026-08-18 S4-R2; S4-R3; S8-R3; S8-R4; renamed to Labor Delta per SV-9071)</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr"/>
@@ -1273,14 +1273,14 @@
 · If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 · If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S4-R5), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R5), read on 18 August 2026.
 Last checked against build v3.5-4795eee on 8/10/2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8967)</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 Story 4 S4-R5 (+ context note))</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 Story 4 S4-R5 (+ context note))</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
@@ -1325,13 +1325,13 @@
 2. The badge is color-coded per the application's standard status colors.
 3. The label text is always present, so color is never the sole signal of the status.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S4-R6, S10-R8), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R6, S10-R8), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 Story 4 S4-R6 + Story 10 S10-R8 — S4-R6 CLOSES the five status labels verbatim ("Estimate" ... "Complete") and the label-not-colour rule; so the closed list IS the requirement)</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 Story 4 S4-R6 + Story 10 S10-R8 — S4-R6 CLOSES the five status labels verbatim ("Estimate" ... "Complete") and the label-not-colour rule; so the closed list IS the requirement)</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr"/>
@@ -1380,13 +1380,13 @@
 5. Note for the tester: the field is labelled VIN. For assets that are not vehicles (for example a generator), this is the unit's serial number.
 Note: this report used to show "(no unit #)" on the first line when a work order had no unit number, and "— no VIN —" for a missing VIN. Both placeholders were changed (Chris Ward, 2026-08-14): a missing unit number now shows the VIN alone on one line, and a missing VIN now shows "Unknown". Follow the new behaviour.
 ---
-This is the expected behaviour as per epic SV-8582 and the Work In Progress report specification version 21 (S4-R7; S4-R8; S4-R9; S4-R10), both read on 17 August 2026. Chris Ward confirmed the two-line asset layout on 5 August 2026 in his answers in this file: https://docs.google.com/spreadsheets/d/1x8cuYJlFsDHalVZZTh156_ZCq2gcOaGY/edit?usp=sharing&amp;ouid=106388879401921597782&amp;rtpof=true&amp;sd=true (read on 11 August 2026); the "(no unit #)"/"— no VIN —" placeholder change is per his 2026-08-14 decision recorded in spec S4-R8.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R7; S4-R8; S4-R9; S4-R10), read on 18 August 2026. Chris Ward confirmed the two-line asset layout on 5 August 2026 in his answers in this file: https://docs.google.com/spreadsheets/d/1x8cuYJlFsDHalVZZTh156_ZCq2gcOaGY/edit?usp=sharing&amp;ouid=106388879401921597782&amp;rtpof=true&amp;sd=true (read on 11 August 2026); the "(no unit #)"/"— no VIN —" placeholder change is per his 2026-08-14 decision recorded in spec S4-R8.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 S4-R7; S4-R8; S4-R9; S4-R10; "(no unit #)" placeholder dropped,VIN alone,missing VIN shows "Unknown" per Chris 2026-08-14)</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 S4-R7; S4-R8; S4-R9; S4-R10; "(no unit #)" placeholder dropped,VIN alone,missing VIN shows "Unknown" per Chris 2026-08-14)</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
@@ -1430,13 +1430,13 @@
           <t>1. The Customer column shows the customer's company name.
 2. The cell is blank when no customer name exists.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S4-R11), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R11), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 Story 4 S4-R11)</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 Story 4 S4-R11)</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr"/>
@@ -1482,13 +1482,13 @@
 2. A same-day work order shows "0 days" and a one-day-old work order shows "1 days".
 3. The value is NOT grammatically pluralized: "1 days" (not "1 day") is the correct, expected rendering.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S4-R12), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R12), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 Story 4 S4-R12; §2 Known Limitations (v1))</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 Story 4 S4-R12; §2 Known Limitations (v1))</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
@@ -1535,13 +1535,13 @@
 2. Otherwise it shows "Xd ago" (for example "3d ago").
 3. A work order with no recorded activity shows "—".
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S4-R13), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R13), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 Story 4 S4-R13)</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 Story 4 S4-R13)</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr"/>
@@ -1597,13 +1597,13 @@
 · If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 · If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582 and the Work In Progress report specification version 21 (S4-R6), both read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R6), read on 18 August 2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8967)</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>SV-8663 (WIP spec v21 2026-08-17 S4; WO number link gating)</t>
+          <t>SV-8663 (WIP spec v22 2026-08-18 S4; WO number link gating)</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
@@ -1650,13 +1650,13 @@
 2. On the work order with a discount, Adjustments shows the discount as a negative amount.
 3. Adjustments is one whole-work-order amount - it is never split into an Earned part and a Remaining part.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and story SV-9282, and the Work In Progress report specification version 21 (S4-R29), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and story SV-9282, and the Work In Progress report specification version 22 (S4-R29), read on 18 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>SV-9282 (WIP spec v21 2026-08-14 S4-R29 — signed net of WO-level fees/discounts,fees positive discounts negative,one whole-WO amount)</t>
+          <t>SV-9282 (WIP spec v22 2026-08-18 S4-R29 — signed net of WO-level fees/discounts,fees positive discounts negative,one whole-WO amount)</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr"/>
@@ -1702,13 +1702,13 @@
 2. Only the Adjustments value and the Total value change.
 3. A line-level fee or discount (one attached to a single line) stays folded into that line's Labor or Parts value and does not appear in Adjustments.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and story SV-9282, and the Work In Progress report specification version 21 (S4-R30), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and story SV-9282, and the Work In Progress report specification version 22 (S4-R30), read on 18 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>SV-9282 (WIP spec v21 2026-08-14 S4-R30 — WO-level amount never allocated into Labor/Parts; line-level stays folded)</t>
+          <t>SV-9282 (WIP spec v22 2026-08-18 S4-R30 — WO-level amount never allocated into Labor/Parts; line-level stays folded)</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
@@ -1754,13 +1754,13 @@
 2. Total is NOT the work order's stored grand total, and it is NOT Earned plus Remaining by itself.
 3. A Total that differs from the work order's own grand total is expected, not a data error.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and story SV-9282, and the Work In Progress report specification version 21 (S4-R21), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and story SV-9282, and the Work In Progress report specification version 22 (S4-R21), read on 18 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>SV-9282 (WIP spec v21 2026-08-14 S4-R21 — Total = Earned + Remaining + Adjustments; not the WO stored grand total)</t>
+          <t>SV-9282 (WIP spec v22 2026-08-18 S4-R21 — Total = Earned + Remaining + Adjustments; not the WO stored grand total)</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr"/>
@@ -1805,13 +1805,13 @@
 2. Earned equals Total minus Adjustments.
 3. Total still equals Earned plus Remaining plus Adjustments.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and story SV-9282, and the Work In Progress report specification version 21 (S4a-R2), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and story SV-9282, and the Work In Progress report specification version 22 (S4a-R2), read on 18 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>SV-9282 (WIP spec v21 2026-08-14 S4a-R2 — Completed tab: Earned = Total - Adjustments,Remaining $0.00)</t>
+          <t>SV-9282 (WIP spec v22 2026-08-18 S4a-R2 — Completed tab: Earned = Total - Adjustments,Remaining $0.00)</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr"/>
@@ -1858,13 +1858,13 @@
 2. A negative value shows a leading minus before the "$" — for example "-$1,234.56".
 3. A genuine zero shows "$0.00".
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S4-R14), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R14), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 Story 4 S4-R14)</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 Story 4 S4-R14)</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr"/>
@@ -1912,13 +1912,13 @@
 2. For the over-clocked line, Labor Earned never exceeds the full quoted value of that line ($400.00 in the example) — the earned share is capped at the quote per line.
 3. With several approved labor lines, Labor Earned is the sum of each line's capped earned share.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S4-R15), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R15), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 Story 4 S4-R15; §4 Terminology (Earned))</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 Story 4 S4-R15; §4 Terminology (Earned))</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr"/>
@@ -1964,13 +1964,13 @@
           <t>1. Labor Remaining equals the total quoted value of the approved labor minus Labor Earned (in the example, $400.00 − $100.00 = $300.00).
 2. Labor Earned + Labor Remaining always equals the total quoted value of the approved labor.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S4-R16), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R16), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 Story 4 S4-R16)</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 Story 4 S4-R16)</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr"/>
@@ -2016,13 +2016,13 @@
           <t>1. Parts Earned equals the sell value of the approved-line parts already received (in the example, $100.00).
 2. Parts not yet received contribute nothing to Parts Earned.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S4-R17), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R17), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 Story 4 S4-R17)</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 Story 4 S4-R17)</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
@@ -2069,13 +2069,13 @@
           <t>1. Parts Remaining equals the sell value of approved-line parts ordered but not yet received (in the example, $100.00).
 2. For the core-charge part, Parts Remaining values the outstanding quantity at its sell price INCLUDING the core charge.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S4-R18), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R18), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 Story 4 S4-R18)</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 Story 4 S4-R18)</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr"/>
@@ -2124,15 +2124,15 @@
 2. Remaining equals Labor Remaining plus Parts Remaining.
 3. Total equals Earned plus Remaining plus Adjustments, so a row's Total matches what invoicing will produce for that work order.
 4. The Total is NOT the work order's stored grand total — it still excludes tax and non-approved lines (the approved fees and discounts are now carried in the Adjustments part), so a difference from the work order's own grand total is EXPECTED, not a data error.
-Note for the tester: an earlier version of this report set Total = Earned + Remaining only. The current Work In Progress report specification (version 21, S4-R21) adds the work order's approved Adjustments, so Total = Earned + Remaining + Adjustments. Follow the current specification.
----
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S4-R19, S4-R20, S4-R21), read on 17 August 2026.
+Note for the tester: an earlier version of this report set Total = Earned + Remaining only. The current Work In Progress report specification (version 22, S4-R21) adds the work order's approved Adjustments, so Total = Earned + Remaining + Adjustments. Follow the current specification.
+---
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R19, S4-R20, S4-R21), read on 18 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 Story 4 S4-R19; S4-R20; S4-R21; §3 Key Decisions)</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 Story 4 S4-R19; S4-R20; S4-R21; §3 Key Decisions)</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr"/>
@@ -2177,13 +2177,13 @@
           <t>1. The work order's Labor/Parts Earned, Labor/Parts Remaining, Earned, Remaining, and Total are unchanged.
 2. Only approved lines (line status authorized or complete) contribute to the report's money — not-yet-approved lines contribute nothing.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S4-R15), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R15), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 Story 4 S4-R15 verbatim 'summed across the work order's approved lines' + §2 Relationship to the work order; §4 Terminology Approved line)</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 Story 4 S4-R15 verbatim 'summed across the work order's approved lines' + §2 Relationship to the work order; §4 Terminology Approved line)</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr"/>
@@ -2234,13 +2234,13 @@
 · If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 · If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582 and the Work In Progress report specification version 21 (S4-R23, S4-R24, S4-E2), both read on 17 August 2026. The column was renamed from "Inv. Hrs" to "Labor Delta" per SV-9071; only the name changed.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R23, S4-R24, S4-E2), read on 18 August 2026. The column was renamed from "Inv. Hrs" to "Labor Delta" per SV-9071; only the name changed.
 AUTOMATION: READY - EXPECT FAIL (SV-8989)</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 S4-R23,S4-R24,S4-E2; heading renamed to Labor Delta per SV-9071)</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 S4-R23,S4-R24,S4-E2; heading renamed to Labor Delta per SV-9071)</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr"/>
@@ -2285,13 +2285,13 @@
           <t>1. Every money column — Labor Earned, Labor Remaining, Parts Earned, Parts Remaining, Earned, Remaining, and Total — shows "$0.00".
 2. The row still appears in the Estimates tab (it is not hidden for having no value).
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S4-E1, S2-R4), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-E1, S2-R4), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 Story 4 S4-E1; Story 2 S2-R4)</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 Story 4 S4-E1; Story 2 S2-R4)</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr"/>
@@ -2339,13 +2339,13 @@
 2. After more time accrues, a refresh shows a larger earned share for that line.
 3. Labor Earned never exceeds the line's full quoted value, no matter how long the clock keeps running — the per-line cap still applies.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S4-R15), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R15), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 Story 4 S4-R15; §4 Terminology (Earned) — spec silent on running clocks; tech-plan-2026-07-29 B1.2 open-clock policy)</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 Story 4 S4-R15; §4 Terminology (Earned) — spec silent on running clocks; tech-plan-2026-07-29 B1.2 open-clock policy)</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr"/>
@@ -2395,13 +2395,13 @@
 4. Parts Earned plus Parts Remaining for that line adds up to the fixed parts portion.
 Note for the tester: on a fixed-price line the customer pays the agreed figure whatever is actually picked or clocked, so the report is expected to show the agreed figure. A difference between the report and the underlying parts or hours is correct here, not a fault.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (the Key Decision on fixed-price valuation added on 2026-08-10 per SV-9028, SV-9035, SV-9040 and SV-9044), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (the Key Decision on fixed-price valuation added on 2026-08-10 per SV-9028, SV-9035, SV-9040 and SV-9044), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 §3 Key Decisions — fixed-price lines are valued at the fixed amounts the customer is billed rather than underlying picked parts or an hourly derivation; added 2026-08-10 per SV-9028; SV-9035; SV-9040; SV-9044)</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 §3 Key Decisions — fixed-price lines are valued at the fixed amounts the customer is billed rather than underlying picked parts or an hourly derivation; added 2026-08-10 per SV-9028; SV-9035; SV-9040; SV-9044)</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr"/>
@@ -2451,13 +2451,13 @@
 4. Once every line is completed the work order has no value left in Remaining.
 Note for the tester: this all-at-once move is expected when there are no invoiced hours to measure progress with. A fixed-price line that DOES have invoiced hours is shared between Earned and Remaining in proportion instead, and that is a different test.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (the Key Decision on fixed-price valuation added on 2026-08-10 per SV-9028, SV-9035, SV-9040 and SV-9044), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (the Key Decision on fixed-price valuation added on 2026-08-10 per SV-9028, SV-9035, SV-9040 and SV-9044), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 §3 Key Decisions — with no invoiced hours the full fixed amount stays in Remaining until the line is completed then moves entirely to Earned; a completed WO never leaves value in Remaining; per SV-9028; SV-9035)</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 §3 Key Decisions — with no invoiced hours the full fixed amount stays in Remaining until the line is completed then moves entirely to Earned; a completed WO never leaves value in Remaining; per SV-9028; SV-9035)</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr"/>
@@ -2506,13 +2506,13 @@
 3. After marking the core Not OK all five figures are again exactly as they were before.
 Note for the tester: deciding a core is handled when the invoice is raised, which is outside this report, so this report is expected not to move at all. If a figure changes when you mark a core, that is a fault worth reporting.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (the Key Decision on core charges added on 2026-08-10 per SV-9057 and SV-9058), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (the Key Decision on core charges added on 2026-08-10 per SV-9057 and SV-9058), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 §3 Key Decisions — a core charge counts in Parts Remaining and Parts Earned at every stage; marking a returned core OK or Not OK never moves the report's figures; added 2026-08-10 per SV-9057; SV-9058)</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 §3 Key Decisions — a core charge counts in Parts Remaining and Parts Earned at every stage; marking a returned core OK or Not OK never moves the report's figures; added 2026-08-10 per SV-9057; SV-9058)</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr"/>
@@ -2555,13 +2555,13 @@
         <is>
           <t>1. The rows are sorted by Days Open, longest-open first (descending).
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S4-R25), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R25), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 Story 4 S4-R25)</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 Story 4 S4-R25)</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr"/>
@@ -2609,13 +2609,13 @@
 3. The third click returns to ascending — there is no third "cleared" state.
 4. Only one column sorts at a time: clicking another header replaces the previous sort.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S4-R26), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R26), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 Story 4 S4-R26)</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 Story 4 S4-R26)</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr"/>
@@ -2665,13 +2665,13 @@
 4. The Asset column sorts by the Unit #.
 5. WO #, Customer, Asset, VIN, Location, and Advisor sort as text.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S4-R9, S4-R27), read on 17 August 2026. Chris Ward confirmed it again on 5 August 2026 in his answers in this file: https://docs.google.com/spreadsheets/d/1x8cuYJlFsDHalVZZTh156_ZCq2gcOaGY/edit?usp=sharing&amp;ouid=106388879401921597782&amp;rtpof=true&amp;sd=true, read on 17 August 2026. It differs from an earlier answer he gave us on 29 July 2026, which we now know was given against a question that described this report incorrectly; we follow his latest word, which agrees with the written description.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R9, S4-R27), read on 18 August 2026. Chris Ward confirmed it again on 5 August 2026 in his answers in this file: https://docs.google.com/spreadsheets/d/1x8cuYJlFsDHalVZZTh156_ZCq2gcOaGY/edit?usp=sharing&amp;ouid=106388879401921597782&amp;rtpof=true&amp;sd=true, read on 17 August 2026. It differs from an earlier answer he gave us on 29 July 2026, which we now know was given against a question that described this report incorrectly; we follow his latest word, which agrees with the written description.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 Story 4 S4-R27; S4-R9 - Asset sort key RE-RULED to the VIN chain (VIN -&gt; Unit # -&gt; plate) by Chris Ward answer 2026-07-29 [newest-wins]; supersedes video P24 serial ruling AND the spec's 'sorts by unit number' rule)</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 Story 4 S4-R27; S4-R9 - Asset sort key RE-RULED to the VIN chain (VIN -&gt; Unit # -&gt; plate) by Chris Ward answer 2026-07-29 [newest-wins]; supersedes video P24 serial ruling AND the spec's 'sorts by unit number' rule)</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr"/>
@@ -2717,13 +2717,13 @@
 2. The Totals row stays pinned at the bottom, out of the sort.
 3. The other tab's order is not changed by the first tab's sort action.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S4-R28), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R28), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 Story 4 S4-R28)</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 Story 4 S4-R28)</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr"/>
@@ -2768,13 +2768,13 @@
 2. There is no Adjustments figure in the summary strip.
 3. Work-order-level fees and discounts are carried only by the Adjustments column and the per-tab Totals row, not by a summary figure.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and story SV-9282, and the Work In Progress report specification version 21 (S5-R1, S5-R13), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and story SV-9282, and the Work In Progress report specification version 22 (S5-R1, S5-R13), read on 18 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>SV-9282 (WIP spec v21 2026-08-14 S5-R1; S5-R13 — seven summary figures,no Adjustments tile (S5-R13 reverses the 2026-08-12 muted figure))</t>
+          <t>SV-9282 (WIP spec v22 2026-08-18 S5-R1; S5-R13 — seven summary figures,no Adjustments tile (S5-R13 reverses the 2026-08-12 muted figure))</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr"/>
@@ -2818,13 +2818,13 @@
           <t>1. The strip shows seven figures, in this order: Total Earned, Total Remaining, Not Started, Started — Earned, Started — Remaining, Ready to Invoice, and Estimates.
 2. Every figure shows US-dollar currency with a leading "$", two decimals, and thousands separators.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S5-R1, S5-R10), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S5-R1, S5-R10), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>SV-8661 (WIP spec v21 2026-08-17 Story 5 S5-R1; S5-R10 — S5-R1 CLOSES the seven figures and their order verbatim and S5-R10 closes the currency format; so the closed lists ARE the requirement)</t>
+          <t>SV-8661 (WIP spec v22 2026-08-18 Story 5 S5-R1; S5-R10 — S5-R1 CLOSES the seven figures and their order verbatim and S5-R10 closes the currency format; so the closed lists ARE the requirement)</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr"/>
@@ -2918,13 +2918,13 @@
         <is>
           <t>1. Total Remaining equals Not Started plus Started — Remaining, to the cent.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S5-R3), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S5-R3), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>SV-8661 (WIP spec v21 2026-08-17 Story 5 S5-R3)</t>
+          <t>SV-8661 (WIP spec v22 2026-08-18 Story 5 S5-R3)</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr"/>
@@ -2971,13 +2971,13 @@
 2. Started — Earned equals the total Earned of the jobs in the "Approved - Partially Completed" tab, and Started — Remaining equals that tab's total Remaining.
 3. Ready to Invoice equals the total Earned of the jobs in the "Completed" tab.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S5-R4, S5-R5, S5-R6, S5-R7), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S5-R4, S5-R5, S5-R6, S5-R7), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>SV-8661 (WIP spec v21 2026-08-17 Story 5 S5-R4; S5-R5; S5-R6; S5-R7)</t>
+          <t>SV-8661 (WIP spec v22 2026-08-18 Story 5 S5-R4; S5-R5; S5-R6; S5-R7)</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr"/>
@@ -3027,14 +3027,14 @@
 · If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 · If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S5-R8, S5-R9), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S5-R8, S5-R9), read on 18 August 2026.
 Last checked against build v3.5-f77875c on 8/6/2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8988)</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>SV-8661 (WIP spec v21 2026-08-17 Story 5 S5-R8; S5-R9)</t>
+          <t>SV-8661 (WIP spec v22 2026-08-18 Story 5 S5-R8; S5-R9)</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr"/>
@@ -3136,13 +3136,13 @@
 2. It equals the sum of the Adjustments values of the tab's visible jobs.
 3. It uses the same signed money format as the column (fees add, discounts subtract).
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and story SV-9282, and the Work In Progress report specification version 21 (S6-R2), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and story SV-9282, and the Work In Progress report specification version 22 (S6-R2), read on 18 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>SV-9282 (WIP spec v21 2026-08-14 S6-R2 — Totals row sums each visible money column including Adjustments)</t>
+          <t>SV-9282 (WIP spec v22 2026-08-18 S6-R2 — Totals row sums each visible money column including Adjustments)</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr"/>
@@ -3188,13 +3188,13 @@
 2. The Totals row's Total cell is pinned far right and shown in bold, matching the column.
 3. The Totals row uses the same number formats as the data rows.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S6-R1, S6-R4, S6-R5), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S6-R1, S6-R4, S6-R5), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>SV-8662 (WIP spec v21 2026-08-17 Story 6 S6-R1; S6-R4; S6-R5)</t>
+          <t>SV-8662 (WIP spec v22 2026-08-18 Story 6 S6-R1; S6-R4; S6-R5)</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr"/>
@@ -3242,13 +3242,13 @@
 3. The Labor Delta total uses the same green (positive) / red (negative) / default (exactly 0.0) coloring as a data row.
 4. Note for the tester: the Labor Delta total can only be checked on screen. On this build a download that includes Labor Delta is refused, so do not try to verify this column from a file.
 ---
-This is the expected behaviour as per epic SV-8582 and the Work In Progress report specification version 21 (S6-R2, S6-R3), both read on 17 August 2026. The column was renamed from "Inv. Hrs" to "Labor Delta" per SV-9071; only the name changed.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S6-R2, S6-R3), read on 18 August 2026. The column was renamed from "Inv. Hrs" to "Labor Delta" per SV-9071; only the name changed.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>SV-8662 (WIP spec v21 2026-08-17 S6-R2,S6-R3; heading renamed to Labor Delta per SV-9071)</t>
+          <t>SV-8662 (WIP spec v22 2026-08-18 S6-R2,S6-R3; heading renamed to Labor Delta per SV-9071)</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr"/>
@@ -3361,14 +3361,14 @@
 · If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 · If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S7-R2, S7-R3), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S7-R2, S7-R3), read on 18 August 2026.
 Last checked against build v3.5-7168d14 on 8/6/2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8969)</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>SV-8663 (WIP spec v21 2026-08-17 Story 7 S7-R2 and S7-R3 — the option list covers every open job in the current scope and not only the loaded rows)</t>
+          <t>SV-8663 (WIP spec v22 2026-08-18 Story 7 S7-R2 and S7-R3 — the option list covers every open job in the current scope and not only the loaded rows)</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr"/>
@@ -3424,14 +3424,14 @@
 · If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 · If it PASSES, the fixes have shipped: tell the QA lead so the tickets can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S7-R4, S7-R5), read on 17 August 2026. Chris Ward confirmed it again on 5 August 2026 in his answers in this file: https://docs.google.com/spreadsheets/d/1x8cuYJlFsDHalVZZTh156_ZCq2gcOaGY/edit?usp=sharing&amp;ouid=106388879401921597782&amp;rtpof=true&amp;sd=true, read on 17 August 2026. It differs from an earlier answer he gave us on 29 July 2026, which we now know was given against a question that described this report incorrectly; we follow his latest word, which agrees with the written description.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S7-R4, S7-R5), read on 18 August 2026. Chris Ward confirmed it again on 5 August 2026 in his answers in this file: https://docs.google.com/spreadsheets/d/1x8cuYJlFsDHalVZZTh156_ZCq2gcOaGY/edit?usp=sharing&amp;ouid=106388879401921597782&amp;rtpof=true&amp;sd=true, read on 17 August 2026. It differs from an earlier answer he gave us on 29 July 2026, which we now know was given against a question that described this report incorrectly; we follow his latest word, which agrees with the written description.
 Last checked against build v3.5-f77875c on 8/6/2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8908, SV-8968)</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>SV-8663 (WIP spec v21 2026-08-17 Story 7 S7-R4 and S7-R5 — the option list covers every asset on every open job in the current scope; option text and match fields per Chris Ward answer 2026-07-29)</t>
+          <t>SV-8663 (WIP spec v22 2026-08-18 Story 7 S7-R4 and S7-R5 — the option list covers every asset on every open job in the current scope; option text and match fields per Chris Ward answer 2026-07-29)</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr"/>
@@ -3477,13 +3477,13 @@
 4. This is the shared "as of" date control that the Inventory Value report also uses.
 Note: the Work In Progress report used to offer a date range with ready-made periods (This Week, This Month and so on) and a build-your-own range. That was replaced by a single "as of" date, a product decision by Chris Ward: work in progress is a point-in-time position, so a range over it would state something the number cannot mean. Follow the single "as of" date and do not look for the old presets or range.
 ---
-This is the expected behaviour as per epic SV-8582 and the Work In Progress report specification version 21 (S7-R6; S7-R8), both read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S7-R6; S7-R8), read on 18 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>SV-9214 (WIP spec v21 2026-08-17 S7-R6; S7-R8; single as-of date replaces the date-range control per Chris 2026-08-13)</t>
+          <t>SV-9214 (WIP spec v22 2026-08-18 S7-R6; S7-R8; single as-of date replaces the date-range control per Chris 2026-08-13)</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr"/>
@@ -3529,13 +3529,13 @@
 3. For today's date the report reads the live open work orders. For an earlier day it reconstructs the position from the nightly snapshot; if no snapshot exists for the selected day it names the nearest earlier recorded day it is showing, and if no snapshot exists at or before that day it says no snapshot is available for that date and shows no rows.
 Note: the Work In Progress report used to offer a date range with ready-made periods (This Week, This Month and so on) and a build-your-own range. That was replaced by a single "as of" date, a product decision by Chris Ward: work in progress is a point-in-time position, so a range over it would state something the number cannot mean. Follow the single "as of" date and do not look for the old presets or range.
 ---
-This is the expected behaviour as per epic SV-8582 and the Work In Progress report specification version 21 (S7-R7; S7-R8a; S2-R6), both read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S7-R7; S7-R8a; S2-R6), read on 18 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>SV-9214 (WIP spec v21 2026-08-17 S7-R7; S7-R8a; S2-R6; single as-of date replaces the date-range control per Chris 2026-08-13)</t>
+          <t>SV-9214 (WIP spec v22 2026-08-18 S7-R7; S7-R8a; S2-R6; single as-of date replaces the date-range control per Chris 2026-08-13)</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr"/>
@@ -3585,13 +3585,13 @@
 3. Selecting one, several, or all locations reloads the report scoped to that set (rows from the added location appear).
 4. For a user with access to only one location the Location filter is NOT shown at all — the report simply shows that one location's work orders.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S7-R9, S7-R10), read on 17 August 2026. Chris Ward confirmed this on 8/5/2026 in his answers in this file: https://docs.google.com/spreadsheets/d/1x8cuYJlFsDHalVZZTh156_ZCq2gcOaGY/edit?usp=sharing&amp;ouid=106388879401921597782&amp;rtpof=true&amp;sd=true, read on 17 August 2026
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S7-R9, S7-R10), read on 18 August 2026. Chris Ward confirmed this on 8/5/2026 in his answers in this file: https://docs.google.com/spreadsheets/d/1x8cuYJlFsDHalVZZTh156_ZCq2gcOaGY/edit?usp=sharing&amp;ouid=106388879401921597782&amp;rtpof=true&amp;sd=true, read on 17 August 2026
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>SV-8663 (WIP spec v21 2026-08-17 Story 7 S7-R9; S7-R10 + on-screen location-scope indicator; spec v21 2026-08-17; single-location filter HIDDEN per Chris Ward answer 2026-07-31 Q1=A)</t>
+          <t>SV-8663 (WIP spec v22 2026-08-18 Story 7 S7-R9; S7-R10 + on-screen location-scope indicator; spec v22 2026-08-18; single-location filter HIDDEN per Chris Ward answer 2026-07-31 Q1=A)</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr"/>
@@ -3637,13 +3637,13 @@
 2. If the selection resolves to none, the report falls back to the user's currently active location rather than showing everything or erroring.
 3. A saved selection that no longer resolves also falls back to the active location.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S7-R11, S8-R8), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S7-R11, S8-R8), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>SV-8663 (WIP spec v21 2026-08-17 Story 7 S7-R11; Story 8 S8-R8)</t>
+          <t>SV-8663 (WIP spec v22 2026-08-18 Story 7 S7-R11; Story 8 S8-R8)</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr"/>
@@ -3693,14 +3693,14 @@
 · If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 · If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S7-R12, S7-N1, S5-R11, S6-R6), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S7-R12, S7-N1, S5-R11, S6-R6), read on 18 August 2026.
 Last checked against build v3.5-7168d14 on 8/6/2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8968)</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>SV-8663 (WIP spec v21 2026-08-17 Story 7 S7-R12; S7-N1; Story 5 S5-R11; Story 6 S6-R6; §3 Key Decisions)</t>
+          <t>SV-8663 (WIP spec v22 2026-08-18 Story 7 S7-R12; S7-N1; Story 5 S5-R11; Story 6 S6-R6; §3 Key Decisions)</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr"/>
@@ -3759,14 +3759,14 @@
 - If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 - If it PASSES, the fix has shipped: tell the QA lead so this note can be removed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S7-R13, S7-R14, S4-R3, S9-E1, S10-R5a), read on 17 August 2026. Chris Ward confirmed this same access-gated, switchable rule in his answers of 8/10/2026, in this file: build/report-suite/chris-answers-2026-08-10/ - his answer and the specification agree, so the earlier note saying the description contradicted itself no longer applies.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S7-R13, S7-R14, S4-R3, S9-E1, S10-R5a), read on 18 August 2026. Chris Ward confirmed this same access-gated, switchable rule in his answers of 8/10/2026, in this file: build/report-suite/chris-answers-2026-08-10/ - his answer and the specification agree, so the earlier note saying the description contradicted itself no longer applies.
 Last checked against build v3.5-4795eee on 8/10/2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8954)</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>SV-8660; SV-8664 (WIP spec v21 2026-08-17 S7-R13; S7-R14; S4-R3; S9-E1; S10-R5a - access-gated toggleable Location column; one location per work-order row so never "Multiple"; headed "Branch" in downloads; constant-width filter)</t>
+          <t>SV-8660; SV-8664 (WIP spec v22 2026-08-18 S7-R13; S7-R14; S4-R3; S9-E1; S10-R5a - access-gated toggleable Location column; one location per work-order row so never "Multiple"; headed "Branch" in downloads; constant-width filter)</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr"/>
@@ -3812,13 +3812,13 @@
 2. Toggling a column off hides it from the table; toggling it on shows it again.
 3. The Total column is always shown and cannot be turned off — it is not offered in the control at all.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S8-R1, S8-R2), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S8-R1, S8-R2), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>SV-8664 (WIP spec v21 2026-08-17 Story 8 S8-R1; S8-R2)</t>
+          <t>SV-8664 (WIP spec v22 2026-08-18 Story 8 S8-R1; S8-R2)</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr"/>
@@ -3864,13 +3864,13 @@
 2. Total is always the last column.
 3. The column selection applies to every tab at once — all four tabs show the same set of columns.
 ---
-This is the expected behaviour as per epic SV-8582 and the Work In Progress report specification version 21 (S4-R1; S8-R7), both read on 17 August 2026. The column was renamed from "Inv. Hrs" to "Labor Delta" per SV-9071; only the name changed.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R1; S8-R7), read on 18 August 2026. The column was renamed from "Inv. Hrs" to "Labor Delta" per SV-9071; only the name changed.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>SV-8664 (WIP spec v21 2026-08-17 S4-R1; S8-R7; renamed to Labor Delta per SV-9071)</t>
+          <t>SV-8664 (WIP spec v22 2026-08-18 S4-R1; S8-R7; renamed to Labor Delta per SV-9071)</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr"/>
@@ -3966,13 +3966,13 @@
           <t>1. The report loads normally — the invalid saved value falls back to that setting's default rather than breaking the view.
 2. All other saved settings are still restored.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S8-R8), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S8-R8), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>SV-8664 (WIP spec v21 2026-08-17 Story 8 S8-R8)</t>
+          <t>SV-8664 (WIP spec v22 2026-08-18 Story 8 S8-R8)</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr"/>
@@ -4025,13 +4025,13 @@
 - If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 - If it PASSES, the fix has shipped: tell the QA lead so this note can be removed.
 ---
-This is the expected behaviour as per epic SV-8582 and the Work In Progress report specification version 21 (S8-R7), both read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S8-R7), read on 18 August 2026.
 AUTOMATION: HOLD - the build does not follow the ratified Location rule; the defect is written up in DEFECTS-FOR-PERMISSION.md and needs the QA lead's permission before a ticket exists to point at</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>SV-8664 (WIP spec v21 2026-08-17 S8-R7; per-column persistence remembers the as-of date)</t>
+          <t>SV-8664 (WIP spec v22 2026-08-18 S8-R7; per-column persistence remembers the as-of date)</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr"/>
@@ -4132,13 +4132,13 @@
 4. Each download (PDF and CSV) carries a "Locations:" line naming the location(s) the report was scoped to.
 5. Note for the tester: the file carries the Location column whenever it is showing on screen. In the file it is headed "Branch", not "Location".
 ---
-This is the expected behaviour as per epic SV-8582 and the Work In Progress report specification version 21 (S9-R3; S9-R10a), both read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S9-R3; S9-R10a), read on 18 August 2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8907)</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>SV-8665 (WIP spec v21 2026-08-17 S9-R3; S9-R10a; downloads honor the as-of date; heading renamed to Labor Delta per SV-9071)</t>
+          <t>SV-8665 (WIP spec v22 2026-08-18 S9-R3; S9-R10a; downloads honor the as-of date; heading renamed to Labor Delta per SV-9071)</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr"/>
@@ -4186,13 +4186,13 @@
 2. In the CSV, a money value containing a comma (a thousands separator) is enclosed in double-quotes per standard CSV rules.
 3. A value without a comma is written unquoted.
 ---
-This is the expected behaviour as per epic SV-8582 and the Work In Progress report specification version 21 (S9-R5, S9-R6), both read on 17 August 2026. The column was renamed from "Inv. Hrs" to "Labor Delta" per SV-9071; only the name changed.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S9-R5, S9-R6), read on 18 August 2026. The column was renamed from "Inv. Hrs" to "Labor Delta" per SV-9071; only the name changed.
 AUTOMATION: READY - EXPECT FAIL (SV-8907)</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>SV-8665 (WIP spec v21 2026-08-17 S9-R5,S9-R6; heading renamed to Labor Delta per SV-9071)</t>
+          <t>SV-8665 (WIP spec v22 2026-08-18 S9-R5,S9-R6; heading renamed to Labor Delta per SV-9071)</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr"/>
@@ -4236,13 +4236,13 @@
           <t>1. In the PDF, Labor Delta keeps the green (positive) / red (negative) coloring.
 2. In the CSV, the Labor Delta column is monochrome — plain signed numbers with no color or markup.
 ---
-This is the expected behaviour as per epic SV-8582 and the Work In Progress report specification version 21 (S9-R7), both read on 17 August 2026. The column was renamed from "Inv. Hrs" to "Labor Delta" per SV-9071; only the name changed.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S9-R7), read on 18 August 2026. The column was renamed from "Inv. Hrs" to "Labor Delta" per SV-9071; only the name changed.
 AUTOMATION: READY - EXPECT FAIL (SV-8907)</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>SV-8665 (WIP spec v21 2026-08-17 S9-R7; heading renamed to Labor Delta per SV-9071)</t>
+          <t>SV-8665 (WIP spec v22 2026-08-18 S9-R7; heading renamed to Labor Delta per SV-9071)</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr"/>
@@ -4287,13 +4287,13 @@
           <t>1. In the download, Days Open is the whole number of days as of the moment the file is generated.
 2. Because the screen computes Days Open live while the file freezes it at generation time, the file can legitimately show a day count one higher than the screen it was generated from — that difference is EXPECTED, not a defect.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S9-R8), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S9-R8), read on 18 August 2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8907)</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>SV-8665 (WIP spec v21 2026-08-17 Story 9 S9-R8; Story 4 context note (Days Open live vs frozen))</t>
+          <t>SV-8665 (WIP spec v22 2026-08-18 Story 9 S9-R8; Story 4 context note (Days Open live vs frozen))</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr"/>
@@ -4391,13 +4391,13 @@
 3. This on-screen-vs-export label difference is the EXPECTED, documented v1 behavior.
 4. The on-screen Asset cell leads with the Unit #, which is what the export header "Unit" already reflects - so no header change is expected here.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S9-E1), read on 17 August 2026. Chris Ward confirmed it again on 5 August 2026 in his answers in this file: https://docs.google.com/spreadsheets/d/1x8cuYJlFsDHalVZZTh156_ZCq2gcOaGY/edit?usp=sharing&amp;ouid=106388879401921597782&amp;rtpof=true&amp;sd=true, read on 17 August 2026. It differs from an earlier answer he gave us on 29 July 2026, which we now know was given against a question that described this report incorrectly; we follow his latest word, which agrees with the written description.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S9-E1), read on 18 August 2026. Chris Ward confirmed it again on 5 August 2026 in his answers in this file: https://docs.google.com/spreadsheets/d/1x8cuYJlFsDHalVZZTh156_ZCq2gcOaGY/edit?usp=sharing&amp;ouid=106388879401921597782&amp;rtpof=true&amp;sd=true, read on 17 August 2026. It differs from an earlier answer he gave us on 29 July 2026, which we now know was given against a question that described this report incorrectly; we follow his latest word, which agrees with the written description.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>SV-8665 (WIP spec v21 2026-08-17 S9-E1; §2 Known Limitations (v1) - asset identifier RE-RULED to the VIN chain (VIN -&gt; Unit # -&gt; plate) by Chris Ward answer 2026-07-29 [newest-wins]; supersedes video P24 serial ruling; export header text unpinned)</t>
+          <t>SV-8665 (WIP spec v22 2026-08-18 S9-E1; §2 Known Limitations (v1) - asset identifier RE-RULED to the VIN chain (VIN -&gt; Unit # -&gt; plate) by Chris Ward answer 2026-07-29 [newest-wins]; supersedes video P24 serial ruling; export header text unpinned)</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr"/>
@@ -4441,13 +4441,13 @@
           <t>1. The PDF shows the shop logo at the top.
 2. The CSV never includes a logo (plain data only).
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S9-R10), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S9-R10), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>SV-8665 (WIP spec v21 2026-08-17 Story 9 S9-R10)</t>
+          <t>SV-8665 (WIP spec v22 2026-08-18 Story 9 S9-R10)</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr"/>
@@ -4547,13 +4547,13 @@
 4. Note for the tester: on this environment the biggest single tab holds about 114 work orders, so you cannot make this message appear here. Record that and move on.
 Why this test cannot be run here: the download has to be over the size limit before this message can appear, and no tab on this environment comes anywhere near it. On top of that, the Work In Progress download currently fails whenever the tab you are on has any rows in it at all - no file arrives and an error appears - which is a separate problem already reported here: https://shopview.atlassian.net/browse/SV-8907. So there is no way to reach the state this test is about. Leave the test as it is and move on.
 ---
-This is the expected behaviour as per epic SV-8582 and the Work In Progress report specification version 21 (S9-R11), both read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S9-R11), read on 18 August 2026.
 AUTOMATION: HOLD - the over-size refusal cannot be produced on this environment; no tab comes near the size limit</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>SV-8665 (WIP spec v21 2026-08-17 S9-R11; export size-cap message drops the date-range clause on this report per Chris 2026-08-13)</t>
+          <t>SV-8665 (WIP spec v22 2026-08-18 S9-R11; export size-cap message drops the date-range clause on this report per Chris 2026-08-13)</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr"/>
@@ -4600,13 +4600,13 @@
 3. A CSV saved or forwarded later is never ambiguous about which filters produced it: every filter the PDF header names is present in the CSV.
 4. Note for the tester: this is the suite-wide rule that the CSV must name the same filters as the PDF. If your report shows no narrowed filters, widen or narrow one so at least one filter line appears, then compare again.
 ---
-This is the expected behaviour as per epic SV-8582 and the Work In Progress report specification version 21 (S9-R10b), both read on 17 August 2026. S9-R10b is the suite-wide rule (added 2026-08-12, SV-9283) that the CSV carries every filter-summary line the PDF header names.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S9-R10b), read on 18 August 2026. S9-R10b is the suite-wide rule (added 2026-08-12, SV-9283) that the CSV carries every filter-summary line the PDF header names.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>SV-8665 (WIP spec v21 2026-08-17 S9-R10b; suite-wide CSV filter-summary rule SV-9283)</t>
+          <t>SV-8665 (WIP spec v22 2026-08-18 S9-R10b; suite-wide CSV filter-summary rule SV-9283)</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr"/>
@@ -4654,14 +4654,14 @@
 · If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 · If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S10-R1), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S10-R1), read on 18 August 2026.
 Last checked against build v3.5-7168d14 on 8/6/2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8970)</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>SV-8666 (WIP spec v21 2026-08-17 Story 10 S10-R1)</t>
+          <t>SV-8666 (WIP spec v22 2026-08-18 Story 10 S10-R1)</t>
         </is>
       </c>
       <c r="I79" s="2" t="inlineStr"/>
@@ -4705,13 +4705,13 @@
           <t>1. The summary strip appears above the tabs.
 2. It is shown as a bold band delineated by a top and bottom rule — not as a row of separate cards.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S10-R2), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S10-R2), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>SV-8666 (WIP spec v21 2026-08-17 Story 10 S10-R2)</t>
+          <t>SV-8666 (WIP spec v22 2026-08-18 Story 10 S10-R2)</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr"/>
@@ -4755,13 +4755,13 @@
           <t>1. The Total column header is bold and pinned to the far right, matching its cells.
 2. The Total column (header and cells, shown in bold) stays fixed to the right edge while the rest of the columns scroll underneath.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S4-R22, S10-R3), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S4-R22, S10-R3), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>SV-8660 (WIP spec v21 2026-08-17 Story 4 S4-R22; Story 10 S10-R3)</t>
+          <t>SV-8660 (WIP spec v22 2026-08-18 Story 4 S4-R22; Story 10 S10-R3)</t>
         </is>
       </c>
       <c r="I81" s="2" t="inlineStr"/>
@@ -4805,13 +4805,13 @@
           <t>1. The Totals row stays visible at the bottom while the rows scroll.
 2. The report fills the available height and only the active tab's table body scrolls — the page itself does not add a second scrollbar.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S10-R4, S10-R5), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S10-R4, S10-R5), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>SV-8666 (WIP spec v21 2026-08-17 Story 10 S10-R4; S10-R5)</t>
+          <t>SV-8666 (WIP spec v22 2026-08-18 Story 10 S10-R4; S10-R5)</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr"/>
@@ -4861,14 +4861,14 @@
 · If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
 · If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S10-R6), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S10-R6), read on 18 August 2026.
 Last checked against build v3.5-4795eee on 8/10/2026.
 AUTOMATION: READY - EXPECT FAIL (SV-8967)</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>SV-8666 (WIP spec v21 2026-08-17 Story 10 S10-R6)</t>
+          <t>SV-8666 (WIP spec v22 2026-08-18 Story 10 S10-R6)</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr"/>
@@ -4914,13 +4914,13 @@
 2. Its explanation is revealed on focus, not by hover alone.
 3. The explanation text is exposed to assistive technology.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S10-R7, S5-R12), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S10-R7, S5-R12), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>SV-8666 (WIP spec v21 2026-08-17 Story 10 S10-R7; Story 5 S5-R12)</t>
+          <t>SV-8666 (WIP spec v22 2026-08-18 Story 10 S10-R7; Story 5 S5-R12)</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr"/>
@@ -4965,13 +4965,13 @@
           <t>1. The report supports dark mode.
 2. The table, the summary strip, the WO # link, the Labor Delta green/red coloring, and the two-line asset cell all use dark-mode-legible colors meeting contrast.
 ---
-This is the expected behaviour as per epic SV-8582 and the Work In Progress report specification version 21 (S10-R9), both read on 17 August 2026. The column was renamed from "Inv. Hrs" to "Labor Delta" per SV-9071; only the name changed.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S10-R9), read on 18 August 2026. The column was renamed from "Inv. Hrs" to "Labor Delta" per SV-9071; only the name changed.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>SV-8666 (WIP spec v21 2026-08-17 S10-R9; heading renamed to Labor Delta per SV-9071)</t>
+          <t>SV-8666 (WIP spec v22 2026-08-18 S10-R9; heading renamed to Labor Delta per SV-9071)</t>
         </is>
       </c>
       <c r="I85" s="2" t="inlineStr"/>
@@ -5018,13 +5018,13 @@
 3. Confirm live against the design/build: the exact highlight colour is described in the design review as an "amber" glow - confirm the exact colour/shade and the exact glow style (outline, underline or shadow) live before pinning them; do not invent a hex value.
 4. Note for the tester: this is the shared reporting-shell tab treatment, so it looks the same on every report that has tabs.
 ---
-This is the expected behaviour as per epic SV-8582, the reporting-shell story SV-8593, and Chris Ward's design-review decisions of 17 August 2026 (the shell tab styling). The Work In Progress report specification version 21 does not name this visual treatment, so the exact styling is Loom-sourced and is marked for live confirmation above (read on 17 August 2026).
+This is the expected behaviour as per epic SV-8582, the reporting-shell story SV-8593, and Chris Ward's design-review decisions of 17 August 2026 (the shell tab styling). The Work In Progress report specification version 22 does not name this visual treatment, so the exact styling is Loom-sourced and is marked for live confirmation above (read on 18 August 2026).
 AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>SV-8593 (WIP spec v21 2026-08-17; shell tab styling per Chris Ward design review 2026-08-17; exact styling to confirm live)</t>
+          <t>SV-8593 (WIP spec v22 2026-08-18; shell tab styling per Chris Ward design review 2026-08-17; exact styling to confirm live)</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr"/>
@@ -5070,13 +5070,13 @@
 2. The download works with the same permission — the specification allows the one ordinary reports access to cover the report and its downloads, with no new permission for it.
 3. Note for the tester: the specification allows ONE ordinary reports access for all six of these new reports and no per-report permission. If the build demands a separate report permission before this works, mark this Failed and report it — do not change the test.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (Story 1 Prerequisites), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (Story 1 Prerequisites), read on 18 August 2026.
 AUTOMATION: READY</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>SV-8657 (WIP spec v21 2026-08-17 Story 1 Prerequisites — one reports permission for all six ruled by Chris Ward Q2=A + QA lead 2026-08-03 "ONE permission FOR NOW"; the WIP prerequisite now states this outright; so his spec edit is DONE)</t>
+          <t>SV-8657 (WIP spec v22 2026-08-18 Story 1 Prerequisites — one reports permission for all six ruled by Chris Ward Q2=A + QA lead 2026-08-03 "ONE permission FOR NOW"; the WIP prerequisite now states this outright; so his spec edit is DONE)</t>
         </is>
       </c>
       <c r="I87" s="2" t="inlineStr"/>
@@ -5171,13 +5171,13 @@
 2. Historical Adjustments values are NOT recomputed from today's data.
 3. Earned and Remaining on those historical rows are unchanged - their captured values do not move.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and story SV-9282, and the Work In Progress report specification version 21 (S11-R8, S11-R9), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and story SV-9282, and the Work In Progress report specification version 22 (S11-R8, S11-R9), read on 18 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>SV-9282 (WIP spec v21 2026-08-14 S11-R8; S11-R9 — Adjustments captured in its own new snapshot column; no history backfill; missing value read as zero)</t>
+          <t>SV-9282 (WIP spec v22 2026-08-18 S11-R8; S11-R9 — Adjustments captured in its own new snapshot column; no history backfill; missing value read as zero)</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr"/>
@@ -5279,19 +5279,19 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>1. The captured Earned equals the on-screen Earned and the captured Remaining equals the on-screen Remaining, to the cent — the snapshot uses the identical computation for both figures, so the two can never diverge for a given work order on the capture date.
+          <t>1. The captured Earned equals the on-screen Earned and the captured Remaining equals the on-screen Remaining, to the cent — the snapshot uses the identical computation for both figures, so the two can never diverge for a given work order and tab on the capture date.
 2. The captured dollar values are stored to the cent — no rounding to whole dollars and no lost cents.
 ---
 Note for the tester: you cannot check this one from any screen. These figures are written each night by a background process, and nothing in the report reads them back in this version. If you cannot see the figures anywhere, mark this test BLOCKED - do not mark it failed, and do not raise it as a problem.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S11-R3, S11-R5), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S11-R3, S11-R5), read on 18 August 2026.
 Last checked against build v3.5-f77875c on 8/6/2026.
 AUTOMATION: HOLD - the nightly capture is written by a background process and nothing in the product reads it back in this version</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>SV-8667 (WIP spec v21 2026-08-17 Story 11 S11-R3; Story 11 S11-R5)</t>
+          <t>SV-8667 (WIP spec v22 2026-08-18 Story 11 S11-R3; Story 11 S11-R5)</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr"/>
@@ -5341,14 +5341,14 @@
 ---
 Note for the tester: you cannot check this one from any screen. These figures are written each night by a background process, and nothing in the report reads them back in this version. If you cannot see the figures anywhere, mark this test BLOCKED - do not mark it failed, and do not raise it as a problem.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S11-R4, S2-R1), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S11-R4, S2-R1), read on 18 August 2026.
 Last checked against build v3.5-f77875c on 8/6/2026.
 AUTOMATION: HOLD - the nightly capture is written by a background process and nothing in the product reads it back in this version</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>SV-8667 (WIP spec v21 2026-08-17 Story 11 S11-R4; Story 2 S2-R1 (first two conditions))</t>
+          <t>SV-8667 (WIP spec v22 2026-08-18 Story 11 S11-R4; Story 2 S2-R1 (first two conditions))</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr"/>
@@ -5395,14 +5395,14 @@
 ---
 Note for the tester: you cannot check this one from any screen. These figures are written each night by a background process, and nothing in the report reads them back in this version. If you cannot see the figures anywhere, mark this test BLOCKED - do not mark it failed, and do not raise it as a problem.
 ---
-This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 21 (S11-R6, S4-E1), read on 17 August 2026.
+This is the expected behaviour as per epic SV-8582, read on 17 August 2026, and the Work In Progress report specification version 22 (S11-R6, S4-E1), read on 18 August 2026.
 Last checked against build v3.5-f77875c on 8/6/2026.
 AUTOMATION: HOLD - the nightly capture is written by a background process and nothing in the product reads it back in this version</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>SV-8667 (WIP spec v21 2026-08-17 Story 11 S11-R6; Story 4 S4-E1)</t>
+          <t>SV-8667 (WIP spec v22 2026-08-18 Story 11 S11-R6; Story 4 S4-E1)</t>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr"/>

</xml_diff>